<commit_message>
added weight on scale
</commit_message>
<xml_diff>
--- a/owlcms/src/main/resources/templates/weighin/WeighInForm-A4.xlsx
+++ b/owlcms/src/main/resources/templates/weighin/WeighInForm-A4.xlsx
@@ -11,7 +11,7 @@
   </sheets>
   <definedNames>
     <definedName name="_1Excel_BuiltIn_Criteria_1_1">'Starting Weights'!#REF!</definedName>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Starting Weights'!$A$14:$L$14</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Starting Weights'!$A$14:$M$14</definedName>
     <definedName name="AFF.">'Starting Weights'!#REF!</definedName>
     <definedName name="Affiliation">'Starting Weights'!#REF!</definedName>
     <definedName name="Barre">#REF!</definedName>
@@ -20,7 +20,7 @@
     <definedName name="CategoryFilter">'Starting Weights'!#REF!</definedName>
     <definedName name="CLUB">'Starting Weights'!#REF!</definedName>
     <definedName name="Collet">#REF!</definedName>
-    <definedName name="_xlnm.Criteria" localSheetId="0">'Starting Weights'!$A$1:$CO$86</definedName>
+    <definedName name="_xlnm.Criteria" localSheetId="0">'Starting Weights'!$A$1:$CP$86</definedName>
     <definedName name="demandé">'Starting Weights'!#REF!</definedName>
     <definedName name="dernier">'Starting Weights'!#REF!</definedName>
     <definedName name="essais">'Starting Weights'!#REF!</definedName>
@@ -43,18 +43,18 @@
     <definedName name="PeséeGroupFilter">'Starting Weights'!#REF!</definedName>
     <definedName name="PRÉNOM">'Starting Weights'!#REF!</definedName>
     <definedName name="progr.">'Starting Weights'!#REF!</definedName>
-    <definedName name="requestedCJ">'Starting Weights'!$R:$R</definedName>
+    <definedName name="requestedCJ">'Starting Weights'!$S:$S</definedName>
     <definedName name="StartGroupFilter">'Starting Weights'!#REF!</definedName>
     <definedName name="TAS">'Starting Weights'!#REF!</definedName>
     <definedName name="tirage">'Starting Weights'!#REF!</definedName>
-    <definedName name="_xlnm.Print_Area" localSheetId="0">'Starting Weights'!$A:$L</definedName>
+    <definedName name="_xlnm.Print_Area" localSheetId="0">'Starting Weights'!$A:$M</definedName>
   </definedNames>
   <calcPr calcId="0"/>
 </workbook>
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="36" uniqueCount="36">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="37" uniqueCount="37">
   <si>
     <t>${t.get("Competition.competitionName")} :</t>
   </si>
@@ -122,7 +122,7 @@
     <t>${t.get("Results.cleanJerk")}</t>
   </si>
   <si>
-    <t>${t.get("Card.Signature")}</t>
+    <t>${t.get("Jury.Signature")}</t>
   </si>
   <si>
     <t>&lt;jx:forEach items="${athletes}" var="l" varStatus="lifterLoop"&gt;</t>
@@ -162,6 +162,9 @@
   </si>
   <si>
     <t>${session.weighIn2}</t>
+  </si>
+  <si>
+    <t>${t.get("ScaleWeight")}</t>
   </si>
 </sst>
 </file>
@@ -429,7 +432,7 @@
     <xf numFmtId="0" fontId="5" fillId="0" borderId="0" applyBorder="0" applyProtection="0"/>
     <xf numFmtId="0" fontId="4" fillId="0" borderId="0" applyBorder="0" applyProtection="0"/>
   </cellStyleXfs>
-  <cellXfs count="48">
+  <cellXfs count="49">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left"/>
@@ -576,6 +579,10 @@
     </xf>
     <xf numFmtId="49" fontId="9" fillId="0" borderId="5" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
       <alignment vertical="center" wrapText="1"/>
+      <protection locked="0"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="5" xfId="0" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="center" wrapText="1"/>
       <protection locked="0"/>
     </xf>
   </cellXfs>
@@ -856,40 +863,41 @@
   <sheetPr filterMode="1">
     <pageSetUpPr fitToPage="1"/>
   </sheetPr>
-  <dimension ref="A1:V112"/>
+  <dimension ref="A1:W112"/>
   <sheetFormatPr defaultColWidth="11" defaultRowHeight="12.75" ns3:dyDescent="0.2"/>
   <cols>
     <col min="1" max="1" width="4.85546875" customWidth="1"/>
     <col min="2" max="2" width="5.7109375" customWidth="1"/>
     <col min="3" max="3" width="41.140625" customWidth="1"/>
     <col min="4" max="4" width="12.140625" customWidth="1"/>
-    <col min="5" max="5" width="11.42578125" style="6" customWidth="1"/>
-    <col min="6" max="7" width="14.28515625" style="6" customWidth="1"/>
-    <col min="8" max="10" width="12.140625" style="7" customWidth="1"/>
-    <col min="11" max="11" width="11.7109375" style="6" customWidth="1"/>
-    <col min="12" max="12" width="10.85546875" style="6" customWidth="1"/>
-    <col min="13" max="13" width="7.7109375" customWidth="1"/>
-    <col min="14" max="14" width="7" style="8" customWidth="1"/>
-    <col min="15" max="15" width="9.140625" style="6" customWidth="1"/>
-    <col min="16" max="17" width="7.7109375" style="6" customWidth="1"/>
-    <col min="18" max="18" width="7.7109375" customWidth="1"/>
-    <col min="19" max="19" width="6.85546875" style="6" customWidth="1"/>
-    <col min="20" max="20" width="7.7109375" style="6" customWidth="1"/>
-    <col min="21" max="21" width="7" style="6" customWidth="1"/>
-    <col min="22" max="22" width="6.28515625" style="6" customWidth="1"/>
-    <col min="23" max="24" width="11.42578125" customWidth="1"/>
+    <col min="5" max="5" width="12.140625" customWidth="1"/>
+    <col min="6" max="6" width="11.42578125" style="6" customWidth="1"/>
+    <col min="7" max="8" width="14.28515625" style="6" customWidth="1"/>
+    <col min="9" max="11" width="12.140625" style="7" customWidth="1"/>
+    <col min="12" max="12" width="11.7109375" style="6" customWidth="1"/>
+    <col min="13" max="13" width="10.85546875" style="6" customWidth="1"/>
+    <col min="14" max="14" width="7.7109375" customWidth="1"/>
+    <col min="15" max="15" width="7" style="8" customWidth="1"/>
+    <col min="16" max="16" width="9.140625" style="6" customWidth="1"/>
+    <col min="17" max="18" width="7.7109375" style="6" customWidth="1"/>
+    <col min="19" max="19" width="7.7109375" customWidth="1"/>
+    <col min="20" max="20" width="6.85546875" style="6" customWidth="1"/>
+    <col min="21" max="21" width="7.7109375" style="6" customWidth="1"/>
+    <col min="22" max="22" width="7" style="6" customWidth="1"/>
+    <col min="23" max="23" width="6.28515625" style="6" customWidth="1"/>
+    <col min="24" max="25" width="11.42578125" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:20" ht="15.75" customHeight="1" ns3:dyDescent="0.25">
+    <row r="1" spans="1:21" ht="15.75" customHeight="1" ns3:dyDescent="0.25">
       <c r="A1" s="9"/>
       <c r="B1" s="10"/>
       <c r="C1" s="11" t="s">
         <v>0</v>
       </c>
-      <c r="D1" s="5" t="s">
+      <c r="D1" s="5"/>
+      <c r="E1" s="5" t="s">
         <v>1</v>
       </c>
-      <c r="E1" s="5"/>
       <c r="F1" s="5"/>
       <c r="G1" s="5"/>
       <c r="H1" s="5"/>
@@ -897,64 +905,68 @@
       <c r="J1" s="5"/>
       <c r="K1" s="5"/>
       <c r="L1" s="5"/>
-      <c r="N1" s="6"/>
-      <c r="R1" s="6"/>
-    </row>
-    <row r="2" spans="1:20" ht="19.5" customHeight="1" ns3:dyDescent="0.2">
+      <c r="M1" s="5"/>
+      <c r="O1" s="6"/>
+      <c r="S1" s="6"/>
+    </row>
+    <row r="2" spans="1:21" ht="19.5" customHeight="1" ns3:dyDescent="0.2">
       <c r="A2" s="12"/>
       <c r="B2" s="13"/>
       <c r="C2" s="11" t="s">
         <v>2</v>
       </c>
-      <c r="D2" s="14" t="s">
+      <c r="D2" s="14"/>
+      <c r="E2" s="14" t="s">
         <v>3</v>
       </c>
-      <c r="E2" s="15"/>
-      <c r="F2" s="16"/>
+      <c r="F2" s="15"/>
       <c r="G2" s="16"/>
-      <c r="H2" s="17"/>
-      <c r="I2" s="18"/>
+      <c r="H2" s="16"/>
+      <c r="I2" s="17"/>
       <c r="J2" s="18"/>
-      <c r="K2" s="15"/>
+      <c r="K2" s="18"/>
       <c r="L2" s="15"/>
-      <c r="N2" s="6"/>
-      <c r="R2" s="6"/>
-    </row>
-    <row r="3" spans="1:20" ht="19.5" customHeight="1" ns3:dyDescent="0.25">
+      <c r="M2" s="15"/>
+      <c r="O2" s="6"/>
+      <c r="S2" s="6"/>
+    </row>
+    <row r="3" spans="1:21" ht="19.5" customHeight="1" ns3:dyDescent="0.25">
       <c r="A3" s="19"/>
       <c r="C3" s="11" t="s">
         <v>4</v>
       </c>
-      <c r="D3" s="20" t="s">
+      <c r="D3" s="20"/>
+      <c r="E3" s="20" t="s">
         <v>5</v>
       </c>
-      <c r="E3" s="20"/>
       <c r="F3" s="20"/>
       <c r="G3" s="20"/>
-      <c r="H3" s="11"/>
-      <c r="I3"/>
+      <c r="H3" s="20"/>
+      <c r="I3" s="11"/>
       <c r="J3"/>
-      <c r="K3" s="21"/>
+      <c r="K3"/>
       <c r="L3" s="21"/>
-      <c r="N3" s="6"/>
-      <c r="R3" s="6"/>
-    </row>
-    <row r="4" spans="1:20" ht="19.5" customHeight="1" ns3:dyDescent="0.25">
+      <c r="M3" s="21"/>
+      <c r="O3" s="6"/>
+      <c r="S3" s="6"/>
+    </row>
+    <row r="4" spans="1:21" ht="19.5" customHeight="1" ns3:dyDescent="0.25">
       <c r="A4" s="19"/>
       <c r="C4" s="11"/>
       <c r="D4" s="22"/>
       <c r="E4" s="22"/>
       <c r="F4" s="22"/>
       <c r="G4" s="22"/>
-      <c r="H4" s="23"/>
-      <c r="I4" s="11"/>
+      <c r="H4" s="22"/>
+      <c r="I4" s="23"/>
       <c r="J4" s="11"/>
-      <c r="K4"/>
-      <c r="L4" s="21"/>
-      <c r="N4" s="6"/>
-      <c r="R4" s="6"/>
-    </row>
-    <row r="5" spans="1:20" ht="19.5" customHeight="1" ns3:dyDescent="0.3">
+      <c r="K4" s="11"/>
+      <c r="L4"/>
+      <c r="M4" s="21"/>
+      <c r="O4" s="6"/>
+      <c r="S4" s="6"/>
+    </row>
+    <row r="5" spans="1:21" ht="19.5" customHeight="1" ns3:dyDescent="0.3">
       <c r="A5" s="19"/>
       <c r="B5" s="4" t="s">
         <v>6</v>
@@ -968,24 +980,26 @@
       <c r="I5" s="4"/>
       <c r="J5" s="4"/>
       <c r="K5" s="4"/>
-      <c r="L5" s="21"/>
-      <c r="N5" s="6"/>
-      <c r="R5" s="6"/>
-    </row>
-    <row r="6" spans="1:20" ht="19.5" customHeight="1" ns3:dyDescent="0.2">
+      <c r="L5" s="4"/>
+      <c r="M5" s="21"/>
+      <c r="O5" s="6"/>
+      <c r="S5" s="6"/>
+    </row>
+    <row r="6" spans="1:21" ht="19.5" customHeight="1" ns3:dyDescent="0.2">
       <c r="A6" s="24"/>
       <c r="B6" s="25"/>
       <c r="C6" s="26"/>
       <c r="D6" s="26"/>
-      <c r="H6" s="6"/>
-      <c r="K6" s="11"/>
-      <c r="L6" s="27"/>
-      <c r="M6" s="6"/>
+      <c r="E6" s="26"/>
+      <c r="I6" s="6"/>
+      <c r="L6" s="11"/>
+      <c r="M6" s="27"/>
       <c r="N6" s="6"/>
-      <c r="Q6" s="11"/>
-      <c r="R6" s="28"/>
-    </row>
-    <row r="7" spans="1:20" ht="19.5" customHeight="1" ns3:dyDescent="0.2">
+      <c r="O6" s="6"/>
+      <c r="R6" s="11"/>
+      <c r="S6" s="28"/>
+    </row>
+    <row r="7" spans="1:21" ht="19.5" customHeight="1" ns3:dyDescent="0.2">
       <c r="A7" s="29" t="s">
         <v>7</v>
       </c>
@@ -999,18 +1013,19 @@
       <c r="I7" s="31"/>
       <c r="J7" s="31"/>
       <c r="K7" s="31"/>
-      <c r="L7" s="32" t="s">
+      <c r="L7" s="31"/>
+      <c r="M7" s="32" t="s">
         <v>8</v>
       </c>
-      <c r="M7" s="6"/>
-      <c r="R7" s="6"/>
-    </row>
-    <row r="8" spans="1:20" ht="13.5" customHeight="1" ns3:dyDescent="0.2">
+      <c r="N7" s="6"/>
+      <c r="S7" s="6"/>
+    </row>
+    <row r="8" spans="1:21" ht="13.5" customHeight="1" ns3:dyDescent="0.2">
       <c r="A8" t="s">
         <v>9</v>
       </c>
     </row>
-    <row r="9" spans="1:20" ht="25.5" customHeight="1" ns3:dyDescent="0.2">
+    <row r="9" spans="1:21" ht="25.5" customHeight="1" ns3:dyDescent="0.2">
       <c r="A9" s="29" t="s">
         <v>10</v>
       </c>
@@ -1024,17 +1039,18 @@
       <c r="I9" s="31"/>
       <c r="J9" s="31"/>
       <c r="K9" s="31"/>
-      <c r="L9" s="33"/>
-      <c r="M9" s="6"/>
-      <c r="R9" s="6"/>
-    </row>
-    <row r="10" spans="1:20" ht="12.75" customHeight="1" ns3:dyDescent="0.2">
+      <c r="L9" s="31"/>
+      <c r="M9" s="33"/>
+      <c r="N9" s="6"/>
+      <c r="S9" s="6"/>
+    </row>
+    <row r="10" spans="1:21" ht="12.75" customHeight="1" ns3:dyDescent="0.2">
       <c r="A10" t="s">
         <v>11</v>
       </c>
     </row>
-    <row r="11" spans="1:20" ht="6" customHeight="1" ns3:dyDescent="0.2"/>
-    <row r="12" spans="1:20" s="6" customFormat="1" ht="15" customHeight="1" ns3:dyDescent="0.2">
+    <row r="11" spans="1:21" ht="6" customHeight="1" ns3:dyDescent="0.2"/>
+    <row r="12" spans="1:21" s="6" customFormat="1" ht="36" customHeight="1" ns3:dyDescent="0.2">
       <c r="A12" s="34" t="s">
         <v>12</v>
       </c>
@@ -1044,43 +1060,46 @@
       <c r="C12" s="34" t="s">
         <v>14</v>
       </c>
-      <c r="D12" s="34" t="s">
+      <c r="D12" s="48" t="s">
+        <v>36</v>
+      </c>
+      <c r="E12" s="34" t="s">
         <v>15</v>
       </c>
-      <c r="E12" s="34" t="s">
+      <c r="F12" s="34" t="s">
         <v>16</v>
       </c>
-      <c r="F12" s="35" t="s">
+      <c r="G12" s="35" t="s">
         <v>17</v>
       </c>
-      <c r="G12" s="35" t="s">
+      <c r="H12" s="35" t="s">
         <v>18</v>
       </c>
-      <c r="H12" s="36" t="s">
+      <c r="I12" s="36" t="s">
         <v>19</v>
       </c>
-      <c r="I12" s="36" t="s">
+      <c r="J12" s="36" t="s">
         <v>20</v>
       </c>
-      <c r="J12" s="36" t="s">
+      <c r="K12" s="36" t="s">
         <v>21</v>
       </c>
-      <c r="K12" s="3" t="s">
+      <c r="L12" s="3" t="s">
         <v>22</v>
       </c>
-      <c r="L12" s="3"/>
-    </row>
-    <row r="13" spans="1:20" ht="14.25" ns3:dyDescent="0.2">
+      <c r="M12" s="3"/>
+    </row>
+    <row r="13" spans="1:21" ht="14.25" ns3:dyDescent="0.2">
       <c r="A13" t="s">
         <v>23</v>
       </c>
-      <c r="H13"/>
-      <c r="I13" s="37"/>
+      <c r="I13"/>
       <c r="J13" s="37"/>
-      <c r="K13"/>
+      <c r="K13" s="37"/>
       <c r="L13"/>
-    </row>
-    <row r="14" spans="1:20" s="45" customFormat="1" ht="32.25" customHeight="1" ns3:dyDescent="0.2">
+      <c r="M13"/>
+    </row>
+    <row r="14" spans="1:21" s="45" customFormat="1" ht="32.25" customHeight="1" ns3:dyDescent="0.2">
       <c r="A14" s="38" t="s">
         <v>24</v>
       </c>
@@ -1091,351 +1110,449 @@
         <v>26</v>
       </c>
       <c r="D14" s="40"/>
-      <c r="E14" s="41" t="s">
+      <c r="E14" s="40"/>
+      <c r="F14" s="41" t="s">
         <v>27</v>
       </c>
-      <c r="F14" s="42" t="s">
+      <c r="G14" s="42" t="s">
         <v>28</v>
       </c>
-      <c r="G14" s="43" t="s">
+      <c r="H14" s="43" t="s">
         <v>29</v>
       </c>
-      <c r="H14" s="44" t="s">
+      <c r="I14" s="44" t="s">
         <v>30</v>
       </c>
-      <c r="I14" s="44"/>
       <c r="J14" s="44"/>
-      <c r="K14" s="2"/>
+      <c r="K14" s="44"/>
       <c r="L14" s="2"/>
-    </row>
-    <row r="15" spans="1:20" ns3:dyDescent="0.2">
+      <c r="M14" s="2"/>
+    </row>
+    <row r="15" spans="1:21" ns3:dyDescent="0.2">
       <c r="A15" t="s">
         <v>31</v>
       </c>
-      <c r="E15"/>
-    </row>
-    <row r="16" spans="1:20" ns3:dyDescent="0.2">
+      <c r="F15"/>
+    </row>
+    <row r="16" spans="1:21" ns3:dyDescent="0.2">
       <c r="D16" s="6"/>
-      <c r="T16" s="46"/>
-    </row>
-    <row r="17" spans="3:20" ht="33" customHeight="1" ns3:dyDescent="0.2">
+      <c r="E16" s="6"/>
+      <c r="U16" s="46"/>
+    </row>
+    <row r="17" spans="3:21" ht="33" customHeight="1" ns3:dyDescent="0.2">
       <c r="C17" t="s">
         <v>32</v>
       </c>
-      <c r="D17" s="1" t="s">
+      <c r="D17" s="1"/>
+      <c r="E17" s="1" t="s">
         <v>33</v>
       </c>
-      <c r="E17" s="1"/>
       <c r="F17" s="1"/>
       <c r="G17" s="1"/>
       <c r="H17" s="1"/>
-      <c r="T17" s="46"/>
-    </row>
-    <row r="18" spans="3:20" ht="33" customHeight="1" ns3:dyDescent="0.2">
+      <c r="I17" s="1"/>
+      <c r="U17" s="46"/>
+    </row>
+    <row r="18" spans="3:21" ht="33" customHeight="1" ns3:dyDescent="0.2">
       <c r="C18" t="s">
         <v>34</v>
       </c>
-      <c r="D18" s="1" t="s">
+      <c r="D18" s="1"/>
+      <c r="E18" s="1" t="s">
         <v>35</v>
       </c>
-      <c r="E18" s="1"/>
       <c r="F18" s="1"/>
       <c r="G18" s="1"/>
       <c r="H18" s="1"/>
-      <c r="T18" s="46"/>
-    </row>
-    <row r="19" spans="3:20" ns3:dyDescent="0.2">
+      <c r="I18" s="1"/>
+      <c r="U18" s="46"/>
+    </row>
+    <row r="19" spans="3:21" ns3:dyDescent="0.2">
       <c r="D19" s="6"/>
-      <c r="T19" s="46"/>
-    </row>
-    <row r="20" spans="3:20" ns3:dyDescent="0.2">
+      <c r="E19" s="6"/>
+      <c r="U19" s="46"/>
+    </row>
+    <row r="20" spans="3:21" ns3:dyDescent="0.2">
       <c r="D20" s="6"/>
-      <c r="T20" s="46"/>
-    </row>
-    <row r="21" spans="3:20" ns3:dyDescent="0.2">
+      <c r="E20" s="6"/>
+      <c r="U20" s="46"/>
+    </row>
+    <row r="21" spans="3:21" ns3:dyDescent="0.2">
       <c r="D21" s="6"/>
-    </row>
-    <row r="22" spans="3:20" ns3:dyDescent="0.2">
+      <c r="E21" s="6"/>
+    </row>
+    <row r="22" spans="3:21" ns3:dyDescent="0.2">
       <c r="D22" s="6"/>
-    </row>
-    <row r="23" spans="3:20" ns3:dyDescent="0.2">
+      <c r="E22" s="6"/>
+    </row>
+    <row r="23" spans="3:21" ns3:dyDescent="0.2">
       <c r="D23" s="6"/>
-    </row>
-    <row r="24" spans="3:20" ns3:dyDescent="0.2">
+      <c r="E23" s="6"/>
+    </row>
+    <row r="24" spans="3:21" ns3:dyDescent="0.2">
       <c r="D24" s="6"/>
-    </row>
-    <row r="25" spans="3:20" ns3:dyDescent="0.2">
+      <c r="E24" s="6"/>
+    </row>
+    <row r="25" spans="3:21" ns3:dyDescent="0.2">
       <c r="D25" s="6"/>
-    </row>
-    <row r="26" spans="3:20" ns3:dyDescent="0.2">
+      <c r="E25" s="6"/>
+    </row>
+    <row r="26" spans="3:21" ns3:dyDescent="0.2">
       <c r="D26" s="6"/>
-    </row>
-    <row r="27" spans="3:20" ns3:dyDescent="0.2">
+      <c r="E26" s="6"/>
+    </row>
+    <row r="27" spans="3:21" ns3:dyDescent="0.2">
       <c r="D27" s="6"/>
-    </row>
-    <row r="28" spans="3:20" ns3:dyDescent="0.2">
+      <c r="E27" s="6"/>
+    </row>
+    <row r="28" spans="3:21" ns3:dyDescent="0.2">
       <c r="D28" s="6"/>
-    </row>
-    <row r="29" spans="3:20" ns3:dyDescent="0.2">
+      <c r="E28" s="6"/>
+    </row>
+    <row r="29" spans="3:21" ns3:dyDescent="0.2">
       <c r="D29" s="6"/>
-    </row>
-    <row r="30" spans="3:20" ns3:dyDescent="0.2">
+      <c r="E29" s="6"/>
+    </row>
+    <row r="30" spans="3:21" ns3:dyDescent="0.2">
       <c r="D30" s="6"/>
-    </row>
-    <row r="31" spans="3:20" ns3:dyDescent="0.2">
+      <c r="E30" s="6"/>
+    </row>
+    <row r="31" spans="3:21" ns3:dyDescent="0.2">
       <c r="D31" s="6"/>
-    </row>
-    <row r="32" spans="3:20" ns3:dyDescent="0.2">
+      <c r="E31" s="6"/>
+    </row>
+    <row r="32" spans="3:21" ns3:dyDescent="0.2">
       <c r="D32" s="6"/>
-    </row>
-    <row r="33" spans="4:4" ns3:dyDescent="0.2">
+      <c r="E32" s="6"/>
+    </row>
+    <row r="33" spans="4:5" ns3:dyDescent="0.2">
       <c r="D33" s="6"/>
-    </row>
-    <row r="34" spans="4:4" ns3:dyDescent="0.2">
+      <c r="E33" s="6"/>
+    </row>
+    <row r="34" spans="4:5" ns3:dyDescent="0.2">
       <c r="D34" s="6"/>
-    </row>
-    <row r="35" spans="4:4" ns3:dyDescent="0.2">
+      <c r="E34" s="6"/>
+    </row>
+    <row r="35" spans="4:5" ns3:dyDescent="0.2">
       <c r="D35" s="6"/>
-    </row>
-    <row r="36" spans="4:4" ns3:dyDescent="0.2">
+      <c r="E35" s="6"/>
+    </row>
+    <row r="36" spans="4:5" ns3:dyDescent="0.2">
       <c r="D36" s="6"/>
-    </row>
-    <row r="37" spans="4:4" ns3:dyDescent="0.2">
+      <c r="E36" s="6"/>
+    </row>
+    <row r="37" spans="4:5" ns3:dyDescent="0.2">
       <c r="D37" s="6"/>
-    </row>
-    <row r="38" spans="4:4" ns3:dyDescent="0.2">
+      <c r="E37" s="6"/>
+    </row>
+    <row r="38" spans="4:5" ns3:dyDescent="0.2">
       <c r="D38" s="6"/>
-    </row>
-    <row r="39" spans="4:4" ns3:dyDescent="0.2">
+      <c r="E38" s="6"/>
+    </row>
+    <row r="39" spans="4:5" ns3:dyDescent="0.2">
       <c r="D39" s="6"/>
-    </row>
-    <row r="40" spans="4:4" ns3:dyDescent="0.2">
+      <c r="E39" s="6"/>
+    </row>
+    <row r="40" spans="4:5" ns3:dyDescent="0.2">
       <c r="D40" s="6"/>
-    </row>
-    <row r="41" spans="4:4" ns3:dyDescent="0.2">
+      <c r="E40" s="6"/>
+    </row>
+    <row r="41" spans="4:5" ns3:dyDescent="0.2">
       <c r="D41" s="6"/>
-    </row>
-    <row r="42" spans="4:4" ns3:dyDescent="0.2">
+      <c r="E41" s="6"/>
+    </row>
+    <row r="42" spans="4:5" ns3:dyDescent="0.2">
       <c r="D42" s="6"/>
-    </row>
-    <row r="43" spans="4:4" ns3:dyDescent="0.2">
+      <c r="E42" s="6"/>
+    </row>
+    <row r="43" spans="4:5" ns3:dyDescent="0.2">
       <c r="D43" s="6"/>
-    </row>
-    <row r="44" spans="4:4" ns3:dyDescent="0.2">
+      <c r="E43" s="6"/>
+    </row>
+    <row r="44" spans="4:5" ns3:dyDescent="0.2">
       <c r="D44" s="6"/>
-    </row>
-    <row r="45" spans="4:4" ns3:dyDescent="0.2">
+      <c r="E44" s="6"/>
+    </row>
+    <row r="45" spans="4:5" ns3:dyDescent="0.2">
       <c r="D45" s="6"/>
-    </row>
-    <row r="46" spans="4:4" ns3:dyDescent="0.2">
+      <c r="E45" s="6"/>
+    </row>
+    <row r="46" spans="4:5" ns3:dyDescent="0.2">
       <c r="D46" s="6"/>
-    </row>
-    <row r="47" spans="4:4" ns3:dyDescent="0.2">
+      <c r="E46" s="6"/>
+    </row>
+    <row r="47" spans="4:5" ns3:dyDescent="0.2">
       <c r="D47" s="6"/>
-    </row>
-    <row r="48" spans="4:4" ns3:dyDescent="0.2">
+      <c r="E47" s="6"/>
+    </row>
+    <row r="48" spans="4:5" ns3:dyDescent="0.2">
       <c r="D48" s="6"/>
-    </row>
-    <row r="49" spans="4:4" ns3:dyDescent="0.2">
+      <c r="E48" s="6"/>
+    </row>
+    <row r="49" spans="4:5" ns3:dyDescent="0.2">
       <c r="D49" s="6"/>
-    </row>
-    <row r="50" spans="4:4" ns3:dyDescent="0.2">
+      <c r="E49" s="6"/>
+    </row>
+    <row r="50" spans="4:5" ns3:dyDescent="0.2">
       <c r="D50" s="6"/>
-    </row>
-    <row r="51" spans="4:4" ns3:dyDescent="0.2">
+      <c r="E50" s="6"/>
+    </row>
+    <row r="51" spans="4:5" ns3:dyDescent="0.2">
       <c r="D51" s="6"/>
-    </row>
-    <row r="52" spans="4:4" ns3:dyDescent="0.2">
+      <c r="E51" s="6"/>
+    </row>
+    <row r="52" spans="4:5" ns3:dyDescent="0.2">
       <c r="D52" s="6"/>
-    </row>
-    <row r="53" spans="4:4" ns3:dyDescent="0.2">
+      <c r="E52" s="6"/>
+    </row>
+    <row r="53" spans="4:5" ns3:dyDescent="0.2">
       <c r="D53" s="6"/>
-    </row>
-    <row r="54" spans="4:4" ns3:dyDescent="0.2">
+      <c r="E53" s="6"/>
+    </row>
+    <row r="54" spans="4:5" ns3:dyDescent="0.2">
       <c r="D54" s="6"/>
-    </row>
-    <row r="55" spans="4:4" ns3:dyDescent="0.2">
+      <c r="E54" s="6"/>
+    </row>
+    <row r="55" spans="4:5" ns3:dyDescent="0.2">
       <c r="D55" s="6"/>
-    </row>
-    <row r="56" spans="4:4" ns3:dyDescent="0.2">
+      <c r="E55" s="6"/>
+    </row>
+    <row r="56" spans="4:5" ns3:dyDescent="0.2">
       <c r="D56" s="6"/>
-    </row>
-    <row r="57" spans="4:4" ns3:dyDescent="0.2">
+      <c r="E56" s="6"/>
+    </row>
+    <row r="57" spans="4:5" ns3:dyDescent="0.2">
       <c r="D57" s="6"/>
-    </row>
-    <row r="58" spans="4:4" ns3:dyDescent="0.2">
+      <c r="E57" s="6"/>
+    </row>
+    <row r="58" spans="4:5" ns3:dyDescent="0.2">
       <c r="D58" s="6"/>
-    </row>
-    <row r="59" spans="4:4" ns3:dyDescent="0.2">
+      <c r="E58" s="6"/>
+    </row>
+    <row r="59" spans="4:5" ns3:dyDescent="0.2">
       <c r="D59" s="6"/>
-    </row>
-    <row r="60" spans="4:4" ns3:dyDescent="0.2">
+      <c r="E59" s="6"/>
+    </row>
+    <row r="60" spans="4:5" ns3:dyDescent="0.2">
       <c r="D60" s="6"/>
-    </row>
-    <row r="61" spans="4:4" ns3:dyDescent="0.2">
+      <c r="E60" s="6"/>
+    </row>
+    <row r="61" spans="4:5" ns3:dyDescent="0.2">
       <c r="D61" s="6"/>
-    </row>
-    <row r="62" spans="4:4" ns3:dyDescent="0.2">
+      <c r="E61" s="6"/>
+    </row>
+    <row r="62" spans="4:5" ns3:dyDescent="0.2">
       <c r="D62" s="6"/>
-    </row>
-    <row r="63" spans="4:4" ns3:dyDescent="0.2">
+      <c r="E62" s="6"/>
+    </row>
+    <row r="63" spans="4:5" ns3:dyDescent="0.2">
       <c r="D63" s="6"/>
-    </row>
-    <row r="64" spans="4:4" ns3:dyDescent="0.2">
+      <c r="E63" s="6"/>
+    </row>
+    <row r="64" spans="4:5" ns3:dyDescent="0.2">
       <c r="D64" s="6"/>
-    </row>
-    <row r="65" spans="4:4" ns3:dyDescent="0.2">
+      <c r="E64" s="6"/>
+    </row>
+    <row r="65" spans="4:5" ns3:dyDescent="0.2">
       <c r="D65" s="6"/>
-    </row>
-    <row r="66" spans="4:4" ns3:dyDescent="0.2">
+      <c r="E65" s="6"/>
+    </row>
+    <row r="66" spans="4:5" ns3:dyDescent="0.2">
       <c r="D66" s="6"/>
-    </row>
-    <row r="67" spans="4:4" ns3:dyDescent="0.2">
+      <c r="E66" s="6"/>
+    </row>
+    <row r="67" spans="4:5" ns3:dyDescent="0.2">
       <c r="D67" s="6"/>
-    </row>
-    <row r="68" spans="4:4" ns3:dyDescent="0.2">
+      <c r="E67" s="6"/>
+    </row>
+    <row r="68" spans="4:5" ns3:dyDescent="0.2">
       <c r="D68" s="6"/>
-    </row>
-    <row r="69" spans="4:4" ns3:dyDescent="0.2">
+      <c r="E68" s="6"/>
+    </row>
+    <row r="69" spans="4:5" ns3:dyDescent="0.2">
       <c r="D69" s="6"/>
-    </row>
-    <row r="70" spans="4:4" ns3:dyDescent="0.2">
+      <c r="E69" s="6"/>
+    </row>
+    <row r="70" spans="4:5" ns3:dyDescent="0.2">
       <c r="D70" s="6"/>
-    </row>
-    <row r="71" spans="4:4" ns3:dyDescent="0.2">
+      <c r="E70" s="6"/>
+    </row>
+    <row r="71" spans="4:5" ns3:dyDescent="0.2">
       <c r="D71" s="6"/>
-    </row>
-    <row r="72" spans="4:4" ns3:dyDescent="0.2">
+      <c r="E71" s="6"/>
+    </row>
+    <row r="72" spans="4:5" ns3:dyDescent="0.2">
       <c r="D72" s="6"/>
-    </row>
-    <row r="73" spans="4:4" ns3:dyDescent="0.2">
+      <c r="E72" s="6"/>
+    </row>
+    <row r="73" spans="4:5" ns3:dyDescent="0.2">
       <c r="D73" s="6"/>
-    </row>
-    <row r="74" spans="4:4" ns3:dyDescent="0.2">
+      <c r="E73" s="6"/>
+    </row>
+    <row r="74" spans="4:5" ns3:dyDescent="0.2">
       <c r="D74" s="6"/>
-    </row>
-    <row r="75" spans="4:4" ns3:dyDescent="0.2">
+      <c r="E74" s="6"/>
+    </row>
+    <row r="75" spans="4:5" ns3:dyDescent="0.2">
       <c r="D75" s="6"/>
-    </row>
-    <row r="76" spans="4:4" ns3:dyDescent="0.2">
+      <c r="E75" s="6"/>
+    </row>
+    <row r="76" spans="4:5" ns3:dyDescent="0.2">
       <c r="D76" s="6"/>
-    </row>
-    <row r="77" spans="4:4" ns3:dyDescent="0.2">
+      <c r="E76" s="6"/>
+    </row>
+    <row r="77" spans="4:5" ns3:dyDescent="0.2">
       <c r="D77" s="6"/>
-    </row>
-    <row r="78" spans="4:4" ns3:dyDescent="0.2">
+      <c r="E77" s="6"/>
+    </row>
+    <row r="78" spans="4:5" ns3:dyDescent="0.2">
       <c r="D78" s="6"/>
-    </row>
-    <row r="79" spans="4:4" ns3:dyDescent="0.2">
+      <c r="E78" s="6"/>
+    </row>
+    <row r="79" spans="4:5" ns3:dyDescent="0.2">
       <c r="D79" s="6"/>
-    </row>
-    <row r="80" spans="4:4" ns3:dyDescent="0.2">
+      <c r="E79" s="6"/>
+    </row>
+    <row r="80" spans="4:5" ns3:dyDescent="0.2">
       <c r="D80" s="6"/>
-    </row>
-    <row r="81" spans="4:4" ns3:dyDescent="0.2">
+      <c r="E80" s="6"/>
+    </row>
+    <row r="81" spans="4:5" ns3:dyDescent="0.2">
       <c r="D81" s="6"/>
-    </row>
-    <row r="82" spans="4:4" ns3:dyDescent="0.2">
+      <c r="E81" s="6"/>
+    </row>
+    <row r="82" spans="4:5" ns3:dyDescent="0.2">
       <c r="D82" s="6"/>
-    </row>
-    <row r="83" spans="4:4" ns3:dyDescent="0.2">
+      <c r="E82" s="6"/>
+    </row>
+    <row r="83" spans="4:5" ns3:dyDescent="0.2">
       <c r="D83" s="6"/>
-    </row>
-    <row r="84" spans="4:4" ns3:dyDescent="0.2">
+      <c r="E83" s="6"/>
+    </row>
+    <row r="84" spans="4:5" ns3:dyDescent="0.2">
       <c r="D84" s="6"/>
-    </row>
-    <row r="85" spans="4:4" ns3:dyDescent="0.2">
+      <c r="E84" s="6"/>
+    </row>
+    <row r="85" spans="4:5" ns3:dyDescent="0.2">
       <c r="D85" s="6"/>
-    </row>
-    <row r="86" spans="4:4" ns3:dyDescent="0.2">
+      <c r="E85" s="6"/>
+    </row>
+    <row r="86" spans="4:5" ns3:dyDescent="0.2">
       <c r="D86" s="6"/>
-    </row>
-    <row r="87" spans="4:4" ns3:dyDescent="0.2">
+      <c r="E86" s="6"/>
+    </row>
+    <row r="87" spans="4:5" ns3:dyDescent="0.2">
       <c r="D87" s="6"/>
-    </row>
-    <row r="88" spans="4:4" ns3:dyDescent="0.2">
+      <c r="E87" s="6"/>
+    </row>
+    <row r="88" spans="4:5" ns3:dyDescent="0.2">
       <c r="D88" s="6"/>
-    </row>
-    <row r="89" spans="4:4" ns3:dyDescent="0.2">
+      <c r="E88" s="6"/>
+    </row>
+    <row r="89" spans="4:5" ns3:dyDescent="0.2">
       <c r="D89" s="6"/>
-    </row>
-    <row r="90" spans="4:4" ns3:dyDescent="0.2">
+      <c r="E89" s="6"/>
+    </row>
+    <row r="90" spans="4:5" ns3:dyDescent="0.2">
       <c r="D90" s="6"/>
-    </row>
-    <row r="91" spans="4:4" ns3:dyDescent="0.2">
+      <c r="E90" s="6"/>
+    </row>
+    <row r="91" spans="4:5" ns3:dyDescent="0.2">
       <c r="D91" s="6"/>
-    </row>
-    <row r="92" spans="4:4" ns3:dyDescent="0.2">
+      <c r="E91" s="6"/>
+    </row>
+    <row r="92" spans="4:5" ns3:dyDescent="0.2">
       <c r="D92" s="6"/>
-    </row>
-    <row r="93" spans="4:4" ns3:dyDescent="0.2">
+      <c r="E92" s="6"/>
+    </row>
+    <row r="93" spans="4:5" ns3:dyDescent="0.2">
       <c r="D93" s="6"/>
-    </row>
-    <row r="94" spans="4:4" ns3:dyDescent="0.2">
+      <c r="E93" s="6"/>
+    </row>
+    <row r="94" spans="4:5" ns3:dyDescent="0.2">
       <c r="D94" s="6"/>
-    </row>
-    <row r="95" spans="4:4" ns3:dyDescent="0.2">
+      <c r="E94" s="6"/>
+    </row>
+    <row r="95" spans="4:5" ns3:dyDescent="0.2">
       <c r="D95" s="6"/>
-    </row>
-    <row r="96" spans="4:4" ns3:dyDescent="0.2">
+      <c r="E95" s="6"/>
+    </row>
+    <row r="96" spans="4:5" ns3:dyDescent="0.2">
       <c r="D96" s="6"/>
-    </row>
-    <row r="97" spans="4:4" ns3:dyDescent="0.2">
+      <c r="E96" s="6"/>
+    </row>
+    <row r="97" spans="4:5" ns3:dyDescent="0.2">
       <c r="D97" s="6"/>
-    </row>
-    <row r="98" spans="4:4" ns3:dyDescent="0.2">
+      <c r="E97" s="6"/>
+    </row>
+    <row r="98" spans="4:5" ns3:dyDescent="0.2">
       <c r="D98" s="6"/>
-    </row>
-    <row r="99" spans="4:4" ns3:dyDescent="0.2">
+      <c r="E98" s="6"/>
+    </row>
+    <row r="99" spans="4:5" ns3:dyDescent="0.2">
       <c r="D99" s="6"/>
-    </row>
-    <row r="100" spans="4:4" ns3:dyDescent="0.2">
+      <c r="E99" s="6"/>
+    </row>
+    <row r="100" spans="4:5" ns3:dyDescent="0.2">
       <c r="D100" s="6"/>
-    </row>
-    <row r="101" spans="4:4" ns3:dyDescent="0.2">
+      <c r="E100" s="6"/>
+    </row>
+    <row r="101" spans="4:5" ns3:dyDescent="0.2">
       <c r="D101" s="6"/>
-    </row>
-    <row r="102" spans="4:4" ns3:dyDescent="0.2">
+      <c r="E101" s="6"/>
+    </row>
+    <row r="102" spans="4:5" ns3:dyDescent="0.2">
       <c r="D102" s="6"/>
-    </row>
-    <row r="103" spans="4:4" ns3:dyDescent="0.2">
+      <c r="E102" s="6"/>
+    </row>
+    <row r="103" spans="4:5" ns3:dyDescent="0.2">
       <c r="D103" s="6"/>
-    </row>
-    <row r="104" spans="4:4" ns3:dyDescent="0.2">
+      <c r="E103" s="6"/>
+    </row>
+    <row r="104" spans="4:5" ns3:dyDescent="0.2">
       <c r="D104" s="6"/>
-    </row>
-    <row r="105" spans="4:4" ns3:dyDescent="0.2">
+      <c r="E104" s="6"/>
+    </row>
+    <row r="105" spans="4:5" ns3:dyDescent="0.2">
       <c r="D105" s="6"/>
-    </row>
-    <row r="106" spans="4:4" ns3:dyDescent="0.2">
+      <c r="E105" s="6"/>
+    </row>
+    <row r="106" spans="4:5" ns3:dyDescent="0.2">
       <c r="D106" s="6"/>
-    </row>
-    <row r="107" spans="4:4" ns3:dyDescent="0.2">
+      <c r="E106" s="6"/>
+    </row>
+    <row r="107" spans="4:5" ns3:dyDescent="0.2">
       <c r="D107" s="6"/>
-    </row>
-    <row r="108" spans="4:4" ns3:dyDescent="0.2">
+      <c r="E107" s="6"/>
+    </row>
+    <row r="108" spans="4:5" ns3:dyDescent="0.2">
       <c r="D108" s="6"/>
-    </row>
-    <row r="109" spans="4:4" ns3:dyDescent="0.2">
+      <c r="E108" s="6"/>
+    </row>
+    <row r="109" spans="4:5" ns3:dyDescent="0.2">
       <c r="D109" s="6"/>
-    </row>
-    <row r="110" spans="4:4" ns3:dyDescent="0.2">
+      <c r="E109" s="6"/>
+    </row>
+    <row r="110" spans="4:5" ns3:dyDescent="0.2">
       <c r="D110" s="6"/>
-    </row>
-    <row r="111" spans="4:4" ns3:dyDescent="0.2">
+      <c r="E110" s="6"/>
+    </row>
+    <row r="111" spans="4:5" ns3:dyDescent="0.2">
       <c r="D111" s="6"/>
-    </row>
-    <row r="112" spans="4:4" ns3:dyDescent="0.2">
+      <c r="E111" s="6"/>
+    </row>
+    <row r="112" spans="4:5" ns3:dyDescent="0.2">
       <c r="D112" s="6"/>
+      <c r="E112" s="6"/>
     </row>
   </sheetData>
   <mergeCells count="6">
-    <mergeCell ref="D18:H18"/>
-    <mergeCell ref="D1:L1"/>
-    <mergeCell ref="B5:K5"/>
-    <mergeCell ref="K12:L12"/>
-    <mergeCell ref="K14:L14"/>
-    <mergeCell ref="D17:H17"/>
+    <mergeCell ref="E18:I18"/>
+    <mergeCell ref="E1:M1"/>
+    <mergeCell ref="B5:L5"/>
+    <mergeCell ref="L12:M12"/>
+    <mergeCell ref="L14:M14"/>
+    <mergeCell ref="E17:I17"/>
   </mergeCells>
   <pageMargins left="0.31527777777777799" right="0.35416666666666702" top="0.39374999999999999" bottom="0.39374999999999999" header="0.511811023622047" footer="0.511811023622047"/>
   <pageSetup paperSize="9" fitToHeight="0" orientation="portrait" horizontalDpi="300" verticalDpi="300"/>

</xml_diff>

<commit_message>
updated to accomodate the IWF and non-IWF signature requirements
</commit_message>
<xml_diff>
--- a/owlcms/src/main/resources/templates/weighin/WeighInForm-A4.xlsx
+++ b/owlcms/src/main/resources/templates/weighin/WeighInForm-A4.xlsx
@@ -228,7 +228,7 @@
       </patternFill>
     </fill>
   </fills>
-  <borders count="9">
+  <borders count="12">
     <border>
       <left/>
       <right/>
@@ -318,6 +318,24 @@
       <diagonal/>
     </border>
     <border/>
+    <border>
+      <right/>
+      <bottom/>
+    </border>
+    <border>
+      <bottom style="thin">
+        <color rgb="00000000"/>
+      </bottom>
+    </border>
+    <border>
+      <left/>
+      <right/>
+      <top/>
+      <bottom style="thin">
+        <color rgb="00000000"/>
+      </bottom>
+      <diagonal/>
+    </border>
   </borders>
   <cellStyleXfs count="12">
     <xf numFmtId="0" fontId="19" fillId="0" borderId="0"/>
@@ -333,7 +351,7 @@
     <xf numFmtId="0" fontId="5" fillId="0" borderId="0"/>
     <xf numFmtId="0" fontId="4" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="61">
+  <cellXfs count="64">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="left"/>
@@ -518,6 +536,16 @@
       <protection locked="0" hidden="0"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="8" fillId="0" borderId="9" applyAlignment="1" applyProtection="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="left"/>
+      <protection locked="0" hidden="0"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="10" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="right"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="8" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center"/>
+    </xf>
   </cellXfs>
   <cellStyles count="12">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -613,7 +641,7 @@
   <commentList>
     <comment ref="A1" authorId="0" shapeId="0">
       <text>
-        <t>jx:area(lastCell="M14")</t>
+        <t>jx:area(lastCell="M15")</t>
       </text>
     </comment>
     <comment ref="A8" authorId="0" shapeId="0">
@@ -844,22 +872,22 @@
           <t>${t.get("Competition.competitionName")} :</t>
         </is>
       </c>
-      <c r="B1" s="50" t="inlineStr">
+      <c r="B1" s="61" t="inlineStr">
         <is>
           <t>${competition.competitionName}</t>
         </is>
       </c>
-      <c r="C1" s="51" t="n"/>
-      <c r="D1" s="51" t="n"/>
-      <c r="E1" s="51" t="n"/>
-      <c r="F1" s="51" t="n"/>
-      <c r="G1" s="51" t="n"/>
-      <c r="H1" s="51" t="n"/>
-      <c r="I1" s="51" t="n"/>
-      <c r="J1" s="51" t="n"/>
-      <c r="K1" s="51" t="n"/>
-      <c r="L1" s="51" t="n"/>
-      <c r="M1" s="51" t="n"/>
+      <c r="C1" s="27" t="n"/>
+      <c r="D1" s="27" t="n"/>
+      <c r="E1" s="27" t="n"/>
+      <c r="F1" s="27" t="n"/>
+      <c r="G1" s="27" t="n"/>
+      <c r="H1" s="27" t="n"/>
+      <c r="I1" s="27" t="n"/>
+      <c r="J1" s="27" t="n"/>
+      <c r="K1" s="27" t="n"/>
+      <c r="L1" s="27" t="n"/>
+      <c r="M1" s="27" t="n"/>
       <c r="O1" s="6" t="n"/>
       <c r="S1" s="6" t="n"/>
     </row>
@@ -1112,44 +1140,52 @@
       <c r="U12" s="46" t="n"/>
     </row>
     <row r="13" ht="33" customHeight="1">
-      <c r="C13" t="inlineStr">
-        <is>
-          <t>${t.get("Weighin1")}</t>
-        </is>
-      </c>
-      <c r="D13" s="1" t="n"/>
-      <c r="E13" s="1" t="inlineStr">
-        <is>
-          <t>${session.weighIn1}</t>
-        </is>
-      </c>
-      <c r="F13" s="60" t="n"/>
-      <c r="G13" s="60" t="n"/>
-      <c r="H13" s="60" t="n"/>
-      <c r="I13" s="60" t="n"/>
+      <c r="A13" s="49" t="n"/>
+      <c r="B13" s="63" t="inlineStr">
+        <is>
+          <t>${"1"}</t>
+        </is>
+      </c>
+      <c r="C13" s="62" t="n"/>
+      <c r="G13" s="49" t="inlineStr">
+        <is>
+          <t>${t.get("CompetitionSecretary1")}</t>
+        </is>
+      </c>
+      <c r="I13" s="62" t="n"/>
       <c r="U13" s="46" t="n"/>
     </row>
     <row r="14" ht="33" customHeight="1">
-      <c r="C14" t="inlineStr">
-        <is>
-          <t>${t.get("Weighin2")}</t>
-        </is>
-      </c>
-      <c r="D14" s="1" t="n"/>
-      <c r="E14" s="1" t="inlineStr">
-        <is>
-          <t>${session.weighIn2}</t>
-        </is>
-      </c>
-      <c r="F14" s="60" t="n"/>
-      <c r="G14" s="60" t="n"/>
-      <c r="H14" s="60" t="n"/>
-      <c r="I14" s="60" t="n"/>
+      <c r="A14" s="49" t="n"/>
+      <c r="B14" s="63" t="inlineStr">
+        <is>
+          <t>${"2"}</t>
+        </is>
+      </c>
+      <c r="C14" s="62" t="n"/>
+      <c r="G14" s="49" t="inlineStr">
+        <is>
+          <t>${t.get("CompetitionSecretary2")}</t>
+        </is>
+      </c>
+      <c r="I14" s="62" t="n"/>
       <c r="U14" s="46" t="n"/>
     </row>
-    <row r="15">
-      <c r="D15" s="6" t="n"/>
-      <c r="E15" s="6" t="n"/>
+    <row r="15" ht="33" customHeight="1">
+      <c r="A15" s="49" t="n"/>
+      <c r="B15" s="63" t="inlineStr">
+        <is>
+          <t>${"3"}</t>
+        </is>
+      </c>
+      <c r="C15" s="62" t="n"/>
+      <c r="G15" s="55" t="n"/>
+      <c r="H15" s="55" t="n"/>
+      <c r="I15" s="55" t="n"/>
+      <c r="J15" s="55" t="n"/>
+      <c r="K15" s="55" t="n"/>
+      <c r="L15" s="55" t="n"/>
+      <c r="M15" s="55" t="n"/>
       <c r="U15" s="46" t="n"/>
     </row>
     <row r="16">
@@ -1526,13 +1562,18 @@
       <c r="E108" s="6" t="n"/>
     </row>
   </sheetData>
-  <mergeCells count="6">
+  <mergeCells count="11">
+    <mergeCell ref="C13:F13"/>
     <mergeCell ref="L10:M10"/>
     <mergeCell ref="B5:L5"/>
-    <mergeCell ref="E13:I13"/>
+    <mergeCell ref="B1:M1"/>
     <mergeCell ref="L11:M11"/>
-    <mergeCell ref="B1:M1"/>
-    <mergeCell ref="E14:I14"/>
+    <mergeCell ref="G14:H14"/>
+    <mergeCell ref="I13:M13"/>
+    <mergeCell ref="C15:F15"/>
+    <mergeCell ref="C14:F14"/>
+    <mergeCell ref="I14:M14"/>
+    <mergeCell ref="G13:H13"/>
   </mergeCells>
   <pageMargins left="0.315277777777778" right="0.354166666666667" top="0.39375" bottom="0.39375" header="0.511811023622047" footer="0.511811023622047"/>
   <pageSetup orientation="portrait" paperSize="9" fitToHeight="0" horizontalDpi="300" verticalDpi="300"/>

</xml_diff>

<commit_message>
Fix weigh-in form header and signature layout
Header labels move from column A (too narrow, clipped) to B, values to C. Referee signature lines use the Referee1-3 translations instead of bare numbers. Every cell of a signature merge now carries the underline, so Excel draws the full line (it only drew the first cell); the secretary label spans F:H so it is no longer clipped. Applied to all A4/LETTER, horizontal and _x2 variants.

Co-authored-by: Copilot <223556219+Copilot@users.noreply.github.com>
</commit_message>
<xml_diff>
--- a/owlcms/src/main/resources/templates/weighin/WeighInForm-A4.xlsx
+++ b/owlcms/src/main/resources/templates/weighin/WeighInForm-A4.xlsx
@@ -867,17 +867,17 @@
   </cols>
   <sheetData>
     <row r="1" ht="15.75" customHeight="1">
-      <c r="A1" s="49" t="inlineStr">
+      <c r="A1" s="49" t="n"/>
+      <c r="B1" s="49" t="inlineStr">
         <is>
           <t>${t.get("Competition.competitionName")} :</t>
         </is>
       </c>
-      <c r="B1" s="61" t="inlineStr">
+      <c r="C1" s="61" t="inlineStr">
         <is>
           <t>${competition.competitionName}</t>
         </is>
       </c>
-      <c r="C1" s="27" t="n"/>
       <c r="D1" s="27" t="n"/>
       <c r="E1" s="27" t="n"/>
       <c r="F1" s="27" t="n"/>
@@ -892,17 +892,17 @@
       <c r="S1" s="6" t="n"/>
     </row>
     <row r="2" ht="19.5" customHeight="1">
-      <c r="A2" s="49" t="inlineStr">
+      <c r="A2" s="49" t="n"/>
+      <c r="B2" s="49" t="inlineStr">
         <is>
           <t>${t.get("Competition.competitionSite")} :</t>
         </is>
       </c>
-      <c r="B2" s="52" t="inlineStr">
+      <c r="C2" s="52" t="inlineStr">
         <is>
           <t>${competition.competitionSite} ${competition.competitionCity}</t>
         </is>
       </c>
-      <c r="C2" s="49" t="n"/>
       <c r="D2" s="52" t="n"/>
       <c r="E2" s="52" t="n"/>
       <c r="F2" s="53" t="n"/>
@@ -917,17 +917,17 @@
       <c r="S2" s="6" t="n"/>
     </row>
     <row r="3" ht="19.5" customHeight="1">
-      <c r="A3" s="49" t="inlineStr">
+      <c r="A3" s="49" t="n"/>
+      <c r="B3" s="49" t="inlineStr">
         <is>
           <t>${t.get("Competition.competitionDate")} :</t>
         </is>
       </c>
-      <c r="B3" s="56" t="inlineStr">
+      <c r="C3" s="56" t="inlineStr">
         <is>
           <t>${competition.localizedCompetitionDate}</t>
         </is>
       </c>
-      <c r="C3" s="49" t="n"/>
       <c r="D3" s="56" t="n"/>
       <c r="E3" s="56" t="n"/>
       <c r="F3" s="56" t="n"/>
@@ -1141,44 +1141,58 @@
     </row>
     <row r="13" ht="33" customHeight="1">
       <c r="A13" s="49" t="n"/>
-      <c r="B13" s="63" t="inlineStr">
-        <is>
-          <t>${"1"}</t>
+      <c r="B13" s="49" t="inlineStr">
+        <is>
+          <t>${t.get("Referee1")}</t>
         </is>
       </c>
       <c r="C13" s="62" t="n"/>
-      <c r="G13" s="49" t="inlineStr">
+      <c r="D13" s="62" t="n"/>
+      <c r="E13" s="62" t="n"/>
+      <c r="F13" s="49" t="inlineStr">
         <is>
           <t>${t.get("CompetitionSecretary1")}</t>
         </is>
       </c>
       <c r="I13" s="62" t="n"/>
+      <c r="J13" s="62" t="n"/>
+      <c r="K13" s="62" t="n"/>
+      <c r="L13" s="62" t="n"/>
+      <c r="M13" s="62" t="n"/>
       <c r="U13" s="46" t="n"/>
     </row>
     <row r="14" ht="33" customHeight="1">
       <c r="A14" s="49" t="n"/>
-      <c r="B14" s="63" t="inlineStr">
-        <is>
-          <t>${"2"}</t>
+      <c r="B14" s="49" t="inlineStr">
+        <is>
+          <t>${t.get("Referee2")}</t>
         </is>
       </c>
       <c r="C14" s="62" t="n"/>
-      <c r="G14" s="49" t="inlineStr">
+      <c r="D14" s="62" t="n"/>
+      <c r="E14" s="62" t="n"/>
+      <c r="F14" s="49" t="inlineStr">
         <is>
           <t>${t.get("CompetitionSecretary2")}</t>
         </is>
       </c>
       <c r="I14" s="62" t="n"/>
+      <c r="J14" s="62" t="n"/>
+      <c r="K14" s="62" t="n"/>
+      <c r="L14" s="62" t="n"/>
+      <c r="M14" s="62" t="n"/>
       <c r="U14" s="46" t="n"/>
     </row>
     <row r="15" ht="33" customHeight="1">
       <c r="A15" s="49" t="n"/>
-      <c r="B15" s="63" t="inlineStr">
-        <is>
-          <t>${"3"}</t>
+      <c r="B15" s="49" t="inlineStr">
+        <is>
+          <t>${t.get("Referee3")}</t>
         </is>
       </c>
       <c r="C15" s="62" t="n"/>
+      <c r="D15" s="62" t="n"/>
+      <c r="E15" s="62" t="n"/>
       <c r="G15" s="55" t="n"/>
       <c r="H15" s="55" t="n"/>
       <c r="I15" s="55" t="n"/>
@@ -1563,17 +1577,17 @@
     </row>
   </sheetData>
   <mergeCells count="11">
-    <mergeCell ref="C13:F13"/>
+    <mergeCell ref="C13:E13"/>
     <mergeCell ref="L10:M10"/>
     <mergeCell ref="B5:L5"/>
-    <mergeCell ref="B1:M1"/>
+    <mergeCell ref="C1:M1"/>
     <mergeCell ref="L11:M11"/>
-    <mergeCell ref="G14:H14"/>
+    <mergeCell ref="F14:H14"/>
     <mergeCell ref="I13:M13"/>
-    <mergeCell ref="C15:F15"/>
-    <mergeCell ref="C14:F14"/>
+    <mergeCell ref="C15:E15"/>
+    <mergeCell ref="C14:E14"/>
     <mergeCell ref="I14:M14"/>
-    <mergeCell ref="G13:H13"/>
+    <mergeCell ref="F13:H13"/>
   </mergeCells>
   <pageMargins left="0.315277777777778" right="0.354166666666667" top="0.39375" bottom="0.39375" header="0.511811023622047" footer="0.511811023622047"/>
   <pageSetup orientation="portrait" paperSize="9" fitToHeight="0" horizontalDpi="300" verticalDpi="300"/>

</xml_diff>